<commit_message>
working upload analysis and pdf report
</commit_message>
<xml_diff>
--- a/uploads/exampleFile.xlsx
+++ b/uploads/exampleFile.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="18">
   <si>
     <t xml:space="preserve">Order ID</t>
   </si>
@@ -68,9 +68,6 @@
   </si>
   <si>
     <t xml:space="preserve">Mouse</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Headphones</t>
   </si>
   <si>
     <t xml:space="preserve">CPU</t>
@@ -155,12 +152,16 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -290,176 +291,174 @@
   <dimension ref="A1:E10"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="14.65"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="14.65"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="0" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="0" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="0" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="0" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="n">
+      <c r="A2" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="0" t="s">
+      <c r="B2" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="0" t="s">
+      <c r="C2" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D2" s="0" t="n">
+      <c r="D2" s="1" t="n">
         <v>167</v>
       </c>
-      <c r="E2" s="1" t="n">
+      <c r="E2" s="2" t="n">
         <v>46111</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="n">
+      <c r="A3" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="0" t="s">
+      <c r="B3" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C3" s="0" t="s">
+      <c r="C3" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="D3" s="0" t="n">
+      <c r="D3" s="1" t="n">
         <v>6456</v>
       </c>
-      <c r="E3" s="1" t="n">
+      <c r="E3" s="2" t="n">
         <v>46111</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="n">
+      <c r="A4" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="0" t="s">
+      <c r="B4" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C4" s="0" t="s">
+      <c r="C4" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="D4" s="0" t="n">
+      <c r="D4" s="1" t="n">
         <v>534</v>
       </c>
-      <c r="E4" s="1" t="n">
+      <c r="E4" s="2" t="n">
         <v>46111</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="n">
+      <c r="A5" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="0" t="s">
+      <c r="B5" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="C5" s="0" t="s">
+      <c r="C5" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="D5" s="0" t="n">
+      <c r="D5" s="1" t="n">
         <v>1213</v>
       </c>
-      <c r="E5" s="1" t="n">
+      <c r="E5" s="2" t="n">
         <v>46111</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="0" t="n">
+      <c r="A6" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="0" t="s">
+      <c r="B6" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="C6" s="0" t="s">
+      <c r="C6" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="D6" s="0" t="n">
+      <c r="D6" s="1" t="n">
         <v>5654</v>
       </c>
-      <c r="E6" s="1" t="n">
+      <c r="E6" s="2" t="n">
         <v>46111</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="0" t="n">
+      <c r="A7" s="1" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="0" t="s">
+      <c r="B7" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C7" s="0" t="s">
+      <c r="C7" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="D7" s="0" t="n">
+      <c r="D7" s="1" t="n">
         <v>554</v>
       </c>
-      <c r="E7" s="1" t="n">
+      <c r="E7" s="2" t="n">
         <v>46111</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="0" t="n">
+      <c r="A8" s="1" t="n">
         <v>7</v>
       </c>
-      <c r="B8" s="0" t="s">
+      <c r="B8" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C8" s="0" t="s">
+      <c r="C8" s="1"/>
+      <c r="D8" s="1" t="n">
+        <v>8</v>
+      </c>
+      <c r="E8" s="2" t="n">
+        <v>46111</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="1" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C9" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="D8" s="0" t="n">
-        <v>8</v>
-      </c>
-      <c r="E8" s="1" t="n">
-        <v>46111</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="0" t="n">
-        <v>8</v>
-      </c>
-      <c r="B9" s="0" t="s">
-        <v>5</v>
-      </c>
-      <c r="C9" s="0" t="s">
+      <c r="D9" s="1" t="n">
+        <v>234</v>
+      </c>
+      <c r="E9" s="2" t="n">
+        <v>46111</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="1" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C10" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="D9" s="0" t="n">
-        <v>234</v>
-      </c>
-      <c r="E9" s="1" t="n">
-        <v>46111</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="0" t="n">
-        <v>9</v>
-      </c>
-      <c r="B10" s="0" t="s">
-        <v>7</v>
-      </c>
-      <c r="C10" s="0" t="s">
-        <v>18</v>
-      </c>
-      <c r="D10" s="0" t="n">
+      <c r="D10" s="1" t="n">
         <v>745</v>
       </c>
-      <c r="E10" s="1" t="n">
+      <c r="E10" s="2" t="n">
         <v>46111</v>
       </c>
     </row>

</xml_diff>